<commit_message>
presentatie sprint 6 + testplan
</commit_message>
<xml_diff>
--- a/Opleverset/Documentatie/Product backlog.xlsx
+++ b/Opleverset/Documentatie/Product backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtha\Documents\GitHub\Project-5-6---Floating-Farm\Opleverset\Documentatie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E4CA7B6-5AB9-4436-B065-C3914778BA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7990C78E-432B-4D95-BDB9-770221476CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{D2F0FAED-A1B1-4AC7-BF59-91D91F5D52A2}"/>
+    <workbookView xWindow="1050" yWindow="1560" windowWidth="19200" windowHeight="11170" xr2:uid="{D2F0FAED-A1B1-4AC7-BF59-91D91F5D52A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Product backlog" sheetId="1" r:id="rId1"/>

</xml_diff>